<commit_message>
updated output feature with summary of waiting time
</commit_message>
<xml_diff>
--- a/PFP-CC/Example 2 Phase Heuristic/Case and Result.xlsx
+++ b/PFP-CC/Example 2 Phase Heuristic/Case and Result.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\GitHub\Work\PFP-CC\Example 2 Phase Heuristic\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\GitHub\PFP-CC\PFP-CC\Example 2 Phase Heuristic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12EFD26E-257C-4EDC-826B-E5D62D5ADDE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F687528D-1444-4DC4-98C2-2806E5F33C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="17550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example" sheetId="38" r:id="rId1"/>
@@ -982,32 +982,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{735922EC-F40F-4B80-B869-1B97FA0E53B8}">
-  <dimension ref="A1:XED11"/>
+  <dimension ref="A1:XEB11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" customWidth="1"/>
     <col min="2" max="2" width="5.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.5546875" customWidth="1"/>
-    <col min="7" max="7" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.6640625" customWidth="1"/>
     <col min="8" max="8" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.5546875" customWidth="1"/>
-    <col min="17" max="17" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="21" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" customWidth="1"/>
+    <col min="10" max="10" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.5546875" customWidth="1"/>
+    <col min="15" max="15" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="19" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="32.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16358" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16356" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A1" s="18" t="s">
         <v>29</v>
       </c>
@@ -1047,42 +1048,42 @@
       <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="14" t="s">
+      <c r="N1" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="O1" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q1" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="R1" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="S1" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="T1" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="U1" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="V1" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="W1" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="O1" s="14" t="s">
+      <c r="X1" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="P1" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q1" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="R1" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="S1" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="T1" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="U1" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="V1" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="W1" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="X1" s="19" t="s">
-        <v>40</v>
-      </c>
       <c r="Y1" s="13"/>
-      <c r="Z1" s="13"/>
-      <c r="AA1" s="13"/>
+      <c r="Z1" s="15"/>
+      <c r="AA1" s="15"/>
       <c r="AB1" s="15"/>
       <c r="AC1" s="15"/>
       <c r="AD1" s="15"/>
@@ -17412,10 +17413,8 @@
       <c r="XDZ1" s="15"/>
       <c r="XEA1" s="15"/>
       <c r="XEB1" s="15"/>
-      <c r="XEC1" s="15"/>
-      <c r="XED1" s="15"/>
     </row>
-    <row r="2" spans="1:16358" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16356" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -17455,53 +17454,53 @@
       <c r="M2" s="22">
         <v>60</v>
       </c>
-      <c r="N2" s="21" t="str">
-        <f t="shared" ref="N2:N11" si="0">"input"&amp;B2&amp;"-"&amp;E2&amp;"-"&amp;J2&amp;"-"&amp;K2&amp;"-"&amp;L2&amp;"-"&amp;M2&amp;".xlsx"</f>
+      <c r="N2" s="23">
+        <v>1.83248840129923</v>
+      </c>
+      <c r="O2" s="24">
+        <v>0.999999999999996</v>
+      </c>
+      <c r="P2" s="23">
+        <v>0.83248840129923696</v>
+      </c>
+      <c r="Q2" s="25">
+        <v>1.78532687734245</v>
+      </c>
+      <c r="R2" s="25">
+        <v>0.94870312499999998</v>
+      </c>
+      <c r="S2" s="25">
+        <v>0.83662375234245501</v>
+      </c>
+      <c r="T2" s="26">
+        <v>0.236688400000275</v>
+      </c>
+      <c r="U2" s="26">
+        <v>302.90680230000299</v>
+      </c>
+      <c r="V2" s="26">
+        <v>303.14349070000299</v>
+      </c>
+      <c r="W2" s="21" t="str">
+        <f>"input"&amp;B2&amp;"-"&amp;E2&amp;"-"&amp;J2&amp;"-"&amp;K2&amp;"-"&amp;L2&amp;"-"&amp;M2&amp;".xlsx"</f>
         <v>input1-128-1-3-50-60.xlsx</v>
       </c>
-      <c r="O2" s="20" t="str">
-        <f>"P1-alone_P2-FL_"&amp;A2&amp;".xlsx"</f>
-        <v>P1-alone_P2-FL_1.xlsx</v>
-      </c>
-      <c r="P2" s="23">
-        <v>1.83248840129923</v>
-      </c>
-      <c r="Q2" s="24">
-        <v>0.999999999999996</v>
-      </c>
-      <c r="R2" s="23">
-        <v>0.83248840129923696</v>
-      </c>
-      <c r="S2" s="25">
-        <v>1.78532687734245</v>
-      </c>
-      <c r="T2" s="25">
-        <v>0.94870312499999998</v>
-      </c>
-      <c r="U2" s="25">
-        <v>0.83662375234245501</v>
-      </c>
-      <c r="V2" s="26">
-        <v>0.236688400000275</v>
-      </c>
-      <c r="W2" s="26">
-        <v>302.90680230000299</v>
-      </c>
-      <c r="X2" s="26">
-        <v>303.14349070000299</v>
-      </c>
-      <c r="BQ2" s="12"/>
-      <c r="EP2" s="12"/>
-      <c r="EW2" s="12"/>
-      <c r="FA2" s="12"/>
-      <c r="IL2" s="12"/>
-      <c r="LK2" s="12"/>
-      <c r="LR2" s="12"/>
-      <c r="LV2" s="12"/>
+      <c r="X2" s="20" t="str">
+        <f>"IP_vector_alone_2FL_reopt-c"&amp;A2&amp;"c.xlsx"</f>
+        <v>IP_vector_alone_2FL_reopt-c1c.xlsx</v>
+      </c>
+      <c r="BO2" s="12"/>
+      <c r="EN2" s="12"/>
+      <c r="EU2" s="12"/>
+      <c r="EY2" s="12"/>
+      <c r="IJ2" s="12"/>
+      <c r="LI2" s="12"/>
+      <c r="LP2" s="12"/>
+      <c r="LT2" s="12"/>
     </row>
-    <row r="3" spans="1:16358" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16356" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <f t="shared" ref="A3:A11" si="1">A2+1</f>
+        <f t="shared" ref="A3:A11" si="0">A2+1</f>
         <v>2</v>
       </c>
       <c r="B3" s="22">
@@ -17540,53 +17539,53 @@
       <c r="M3" s="22">
         <v>60</v>
       </c>
-      <c r="N3" s="21" t="str">
+      <c r="N3" s="23">
+        <v>1.83248840129923</v>
+      </c>
+      <c r="O3" s="24">
+        <v>0.999999999999994</v>
+      </c>
+      <c r="P3" s="23">
+        <v>0.83248840129923796</v>
+      </c>
+      <c r="Q3" s="25">
+        <v>1.7857538285518999</v>
+      </c>
+      <c r="R3" s="25">
+        <v>0.95043593749999999</v>
+      </c>
+      <c r="S3" s="25">
+        <v>0.83531789105190202</v>
+      </c>
+      <c r="T3" s="26">
+        <v>0.27002849999917</v>
+      </c>
+      <c r="U3" s="26">
+        <v>216.658999699997</v>
+      </c>
+      <c r="V3" s="26">
+        <v>216.929028199996</v>
+      </c>
+      <c r="W3" s="21" t="str">
+        <f>"input"&amp;B3&amp;"-"&amp;E3&amp;"-"&amp;J3&amp;"-"&amp;K3&amp;"-"&amp;L3&amp;"-"&amp;M3&amp;".xlsx"</f>
+        <v>input2-128-1-3-50-60.xlsx</v>
+      </c>
+      <c r="X3" s="20" t="str">
+        <f t="shared" ref="X3:X11" si="1">"IP_vector_alone_2FL_reopt-c"&amp;A3&amp;"c.xlsx"</f>
+        <v>IP_vector_alone_2FL_reopt-c2c.xlsx</v>
+      </c>
+      <c r="BO3" s="12"/>
+      <c r="EN3" s="12"/>
+      <c r="EU3" s="12"/>
+      <c r="EY3" s="12"/>
+      <c r="IJ3" s="12"/>
+      <c r="LI3" s="12"/>
+      <c r="LP3" s="12"/>
+      <c r="LT3" s="12"/>
+    </row>
+    <row r="4" spans="1:16356" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
         <f t="shared" si="0"/>
-        <v>input2-128-1-3-50-60.xlsx</v>
-      </c>
-      <c r="O3" s="20" t="str">
-        <f t="shared" ref="O3:O11" si="2">"P1-alone_P2-FL_"&amp;A3&amp;".xlsx"</f>
-        <v>P1-alone_P2-FL_2.xlsx</v>
-      </c>
-      <c r="P3" s="23">
-        <v>1.83248840129923</v>
-      </c>
-      <c r="Q3" s="24">
-        <v>0.999999999999994</v>
-      </c>
-      <c r="R3" s="23">
-        <v>0.83248840129923796</v>
-      </c>
-      <c r="S3" s="25">
-        <v>1.7857538285518999</v>
-      </c>
-      <c r="T3" s="25">
-        <v>0.95043593749999999</v>
-      </c>
-      <c r="U3" s="25">
-        <v>0.83531789105190202</v>
-      </c>
-      <c r="V3" s="26">
-        <v>0.27002849999917</v>
-      </c>
-      <c r="W3" s="26">
-        <v>216.658999699997</v>
-      </c>
-      <c r="X3" s="26">
-        <v>216.929028199996</v>
-      </c>
-      <c r="BQ3" s="12"/>
-      <c r="EP3" s="12"/>
-      <c r="EW3" s="12"/>
-      <c r="FA3" s="12"/>
-      <c r="IL3" s="12"/>
-      <c r="LK3" s="12"/>
-      <c r="LR3" s="12"/>
-      <c r="LV3" s="12"/>
-    </row>
-    <row r="4" spans="1:16358" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="B4" s="22">
@@ -17625,53 +17624,53 @@
       <c r="M4" s="22">
         <v>60</v>
       </c>
-      <c r="N4" s="21" t="str">
+      <c r="N4" s="23">
+        <v>1.83248840129923</v>
+      </c>
+      <c r="O4" s="24">
+        <v>0.999999999999998</v>
+      </c>
+      <c r="P4" s="23">
+        <v>0.83248840129923796</v>
+      </c>
+      <c r="Q4" s="25">
+        <v>1.78911656138715</v>
+      </c>
+      <c r="R4" s="25">
+        <v>0.95503749999999898</v>
+      </c>
+      <c r="S4" s="25">
+        <v>0.83407906138715604</v>
+      </c>
+      <c r="T4" s="26">
+        <v>0.29539320000185398</v>
+      </c>
+      <c r="U4" s="26">
+        <v>238.950062299991</v>
+      </c>
+      <c r="V4" s="26">
+        <v>239.245455499993</v>
+      </c>
+      <c r="W4" s="21" t="str">
+        <f>"input"&amp;B4&amp;"-"&amp;E4&amp;"-"&amp;J4&amp;"-"&amp;K4&amp;"-"&amp;L4&amp;"-"&amp;M4&amp;".xlsx"</f>
+        <v>input3-128-1-3-50-60.xlsx</v>
+      </c>
+      <c r="X4" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v>IP_vector_alone_2FL_reopt-c3c.xlsx</v>
+      </c>
+      <c r="BO4" s="12"/>
+      <c r="EN4" s="12"/>
+      <c r="EU4" s="12"/>
+      <c r="EY4" s="12"/>
+      <c r="IJ4" s="12"/>
+      <c r="LI4" s="12"/>
+      <c r="LP4" s="12"/>
+      <c r="LT4" s="12"/>
+    </row>
+    <row r="5" spans="1:16356" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
         <f t="shared" si="0"/>
-        <v>input3-128-1-3-50-60.xlsx</v>
-      </c>
-      <c r="O4" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v>P1-alone_P2-FL_3.xlsx</v>
-      </c>
-      <c r="P4" s="23">
-        <v>1.83248840129923</v>
-      </c>
-      <c r="Q4" s="24">
-        <v>0.999999999999998</v>
-      </c>
-      <c r="R4" s="23">
-        <v>0.83248840129923796</v>
-      </c>
-      <c r="S4" s="25">
-        <v>1.78911656138715</v>
-      </c>
-      <c r="T4" s="25">
-        <v>0.95503749999999898</v>
-      </c>
-      <c r="U4" s="25">
-        <v>0.83407906138715604</v>
-      </c>
-      <c r="V4" s="26">
-        <v>0.29539320000185398</v>
-      </c>
-      <c r="W4" s="26">
-        <v>238.950062299991</v>
-      </c>
-      <c r="X4" s="26">
-        <v>239.245455499993</v>
-      </c>
-      <c r="BQ4" s="12"/>
-      <c r="EP4" s="12"/>
-      <c r="EW4" s="12"/>
-      <c r="FA4" s="12"/>
-      <c r="IL4" s="12"/>
-      <c r="LK4" s="12"/>
-      <c r="LR4" s="12"/>
-      <c r="LV4" s="12"/>
-    </row>
-    <row r="5" spans="1:16358" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="B5" s="22">
@@ -17710,53 +17709,53 @@
       <c r="M5" s="22">
         <v>60</v>
       </c>
-      <c r="N5" s="21" t="str">
+      <c r="N5" s="23">
+        <v>1.833081997151</v>
+      </c>
+      <c r="O5" s="24">
+        <v>0.999999999999994</v>
+      </c>
+      <c r="P5" s="23">
+        <v>0.83308199715100695</v>
+      </c>
+      <c r="Q5" s="25">
+        <v>1.78556931563845</v>
+      </c>
+      <c r="R5" s="25">
+        <v>0.94889843750000102</v>
+      </c>
+      <c r="S5" s="25">
+        <v>0.83667087813845298</v>
+      </c>
+      <c r="T5" s="26">
+        <v>0.39418900000237</v>
+      </c>
+      <c r="U5" s="26">
+        <v>542.80704120000098</v>
+      </c>
+      <c r="V5" s="26">
+        <v>543.20123020000301</v>
+      </c>
+      <c r="W5" s="21" t="str">
+        <f>"input"&amp;B5&amp;"-"&amp;E5&amp;"-"&amp;J5&amp;"-"&amp;K5&amp;"-"&amp;L5&amp;"-"&amp;M5&amp;".xlsx"</f>
+        <v>input4-128-1-3-50-60.xlsx</v>
+      </c>
+      <c r="X5" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v>IP_vector_alone_2FL_reopt-c4c.xlsx</v>
+      </c>
+      <c r="BO5" s="12"/>
+      <c r="EN5" s="12"/>
+      <c r="EU5" s="12"/>
+      <c r="EY5" s="12"/>
+      <c r="IJ5" s="12"/>
+      <c r="LI5" s="12"/>
+      <c r="LP5" s="12"/>
+      <c r="LT5" s="12"/>
+    </row>
+    <row r="6" spans="1:16356" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
         <f t="shared" si="0"/>
-        <v>input4-128-1-3-50-60.xlsx</v>
-      </c>
-      <c r="O5" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v>P1-alone_P2-FL_4.xlsx</v>
-      </c>
-      <c r="P5" s="23">
-        <v>1.833081997151</v>
-      </c>
-      <c r="Q5" s="24">
-        <v>0.999999999999994</v>
-      </c>
-      <c r="R5" s="23">
-        <v>0.83308199715100695</v>
-      </c>
-      <c r="S5" s="25">
-        <v>1.78556931563845</v>
-      </c>
-      <c r="T5" s="25">
-        <v>0.94889843750000102</v>
-      </c>
-      <c r="U5" s="25">
-        <v>0.83667087813845298</v>
-      </c>
-      <c r="V5" s="26">
-        <v>0.39418900000237</v>
-      </c>
-      <c r="W5" s="26">
-        <v>542.80704120000098</v>
-      </c>
-      <c r="X5" s="26">
-        <v>543.20123020000301</v>
-      </c>
-      <c r="BQ5" s="12"/>
-      <c r="EP5" s="12"/>
-      <c r="EW5" s="12"/>
-      <c r="FA5" s="12"/>
-      <c r="IL5" s="12"/>
-      <c r="LK5" s="12"/>
-      <c r="LR5" s="12"/>
-      <c r="LV5" s="12"/>
-    </row>
-    <row r="6" spans="1:16358" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="B6" s="22">
@@ -17795,57 +17794,57 @@
       <c r="M6" s="22">
         <v>60</v>
       </c>
-      <c r="N6" s="21" t="str">
+      <c r="N6" s="23">
+        <v>1.83248840129923</v>
+      </c>
+      <c r="O6" s="24">
+        <v>0.999999999999996</v>
+      </c>
+      <c r="P6" s="23">
+        <v>0.83248840129923796</v>
+      </c>
+      <c r="Q6" s="25">
+        <v>1.7804503939827501</v>
+      </c>
+      <c r="R6" s="25">
+        <v>0.94498906249474501</v>
+      </c>
+      <c r="S6" s="25">
+        <v>0.83546133148801305</v>
+      </c>
+      <c r="T6" s="26">
+        <v>0.35348570000132801</v>
+      </c>
+      <c r="U6" s="26">
+        <v>287.33630029999699</v>
+      </c>
+      <c r="V6" s="26">
+        <v>287.689785999999</v>
+      </c>
+      <c r="W6" s="21" t="str">
+        <f>"input"&amp;B6&amp;"-"&amp;E6&amp;"-"&amp;J6&amp;"-"&amp;K6&amp;"-"&amp;L6&amp;"-"&amp;M6&amp;".xlsx"</f>
+        <v>input5-128-1-3-50-60.xlsx</v>
+      </c>
+      <c r="X6" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v>IP_vector_alone_2FL_reopt-c5c.xlsx</v>
+      </c>
+      <c r="BO6" s="12"/>
+      <c r="EN6" s="12"/>
+      <c r="EU6" s="12"/>
+      <c r="EY6" s="12"/>
+      <c r="FV6" s="12"/>
+      <c r="FX6" s="12"/>
+      <c r="IJ6" s="12"/>
+      <c r="LI6" s="12"/>
+      <c r="LP6" s="12"/>
+      <c r="LT6" s="12"/>
+      <c r="MQ6" s="12"/>
+      <c r="MS6" s="12"/>
+    </row>
+    <row r="7" spans="1:16356" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
         <f t="shared" si="0"/>
-        <v>input5-128-1-3-50-60.xlsx</v>
-      </c>
-      <c r="O6" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v>P1-alone_P2-FL_5.xlsx</v>
-      </c>
-      <c r="P6" s="23">
-        <v>1.83248840129923</v>
-      </c>
-      <c r="Q6" s="24">
-        <v>0.999999999999996</v>
-      </c>
-      <c r="R6" s="23">
-        <v>0.83248840129923796</v>
-      </c>
-      <c r="S6" s="25">
-        <v>1.7804503939827501</v>
-      </c>
-      <c r="T6" s="25">
-        <v>0.94498906249474501</v>
-      </c>
-      <c r="U6" s="25">
-        <v>0.83546133148801305</v>
-      </c>
-      <c r="V6" s="26">
-        <v>0.35348570000132801</v>
-      </c>
-      <c r="W6" s="26">
-        <v>287.33630029999699</v>
-      </c>
-      <c r="X6" s="26">
-        <v>287.689785999999</v>
-      </c>
-      <c r="BQ6" s="12"/>
-      <c r="EP6" s="12"/>
-      <c r="EW6" s="12"/>
-      <c r="FA6" s="12"/>
-      <c r="FX6" s="12"/>
-      <c r="FZ6" s="12"/>
-      <c r="IL6" s="12"/>
-      <c r="LK6" s="12"/>
-      <c r="LR6" s="12"/>
-      <c r="LV6" s="12"/>
-      <c r="MS6" s="12"/>
-      <c r="MU6" s="12"/>
-    </row>
-    <row r="7" spans="1:16358" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="B7" s="22">
@@ -17884,47 +17883,47 @@
       <c r="M7" s="22">
         <v>60</v>
       </c>
-      <c r="N7" s="21" t="str">
+      <c r="N7" s="23">
+        <v>1.83258178117915</v>
+      </c>
+      <c r="O7" s="24">
+        <v>0.999999999999997</v>
+      </c>
+      <c r="P7" s="23">
+        <v>0.83258178117915604</v>
+      </c>
+      <c r="Q7" s="25">
+        <v>1.8202943319324401</v>
+      </c>
+      <c r="R7" s="25">
+        <v>0.97050859374999698</v>
+      </c>
+      <c r="S7" s="25">
+        <v>0.84978573818244496</v>
+      </c>
+      <c r="T7" s="26">
+        <v>0.77009069999621704</v>
+      </c>
+      <c r="U7" s="26">
+        <v>600.751102299997</v>
+      </c>
+      <c r="V7" s="26">
+        <v>601.52119299999299</v>
+      </c>
+      <c r="W7" s="21" t="str">
+        <f>"input"&amp;B7&amp;"-"&amp;E7&amp;"-"&amp;J7&amp;"-"&amp;K7&amp;"-"&amp;L7&amp;"-"&amp;M7&amp;".xlsx"</f>
+        <v>input1-256-1-3-50-60.xlsx</v>
+      </c>
+      <c r="X7" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v>IP_vector_alone_2FL_reopt-c6c.xlsx</v>
+      </c>
+      <c r="BO7" s="12"/>
+      <c r="IJ7" s="12"/>
+    </row>
+    <row r="8" spans="1:16356" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
         <f t="shared" si="0"/>
-        <v>input1-256-1-3-50-60.xlsx</v>
-      </c>
-      <c r="O7" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v>P1-alone_P2-FL_6.xlsx</v>
-      </c>
-      <c r="P7" s="23">
-        <v>1.83258178117915</v>
-      </c>
-      <c r="Q7" s="24">
-        <v>0.999999999999997</v>
-      </c>
-      <c r="R7" s="23">
-        <v>0.83258178117915604</v>
-      </c>
-      <c r="S7" s="25">
-        <v>1.8202943319324401</v>
-      </c>
-      <c r="T7" s="25">
-        <v>0.97050859374999698</v>
-      </c>
-      <c r="U7" s="25">
-        <v>0.84978573818244496</v>
-      </c>
-      <c r="V7" s="26">
-        <v>0.77009069999621704</v>
-      </c>
-      <c r="W7" s="26">
-        <v>600.751102299997</v>
-      </c>
-      <c r="X7" s="26">
-        <v>601.52119299999299</v>
-      </c>
-      <c r="BQ7" s="12"/>
-      <c r="IL7" s="12"/>
-    </row>
-    <row r="8" spans="1:16358" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="B8" s="22">
@@ -17963,53 +17962,53 @@
       <c r="M8" s="22">
         <v>60</v>
       </c>
-      <c r="N8" s="21" t="str">
+      <c r="N8" s="23">
+        <v>1.8324760595354599</v>
+      </c>
+      <c r="O8" s="24">
+        <v>0.999999999999997</v>
+      </c>
+      <c r="P8" s="23">
+        <v>0.83247605953546899</v>
+      </c>
+      <c r="Q8" s="25">
+        <v>1.77752156719893</v>
+      </c>
+      <c r="R8" s="25">
+        <v>0.94110312500000004</v>
+      </c>
+      <c r="S8" s="25">
+        <v>0.83641844219893502</v>
+      </c>
+      <c r="T8" s="26">
+        <v>0.78943180000351199</v>
+      </c>
+      <c r="U8" s="26">
+        <v>599.45193720001396</v>
+      </c>
+      <c r="V8" s="26">
+        <v>600.24136900001702</v>
+      </c>
+      <c r="W8" s="21" t="str">
+        <f>"input"&amp;B8&amp;"-"&amp;E8&amp;"-"&amp;J8&amp;"-"&amp;K8&amp;"-"&amp;L8&amp;"-"&amp;M8&amp;".xlsx"</f>
+        <v>input2-256-1-3-50-60.xlsx</v>
+      </c>
+      <c r="X8" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v>IP_vector_alone_2FL_reopt-c7c.xlsx</v>
+      </c>
+      <c r="BO8" s="12"/>
+      <c r="EN8" s="12"/>
+      <c r="EU8" s="12"/>
+      <c r="EY8" s="12"/>
+      <c r="IJ8" s="12"/>
+      <c r="LI8" s="12"/>
+      <c r="LP8" s="12"/>
+      <c r="LT8" s="12"/>
+    </row>
+    <row r="9" spans="1:16356" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
         <f t="shared" si="0"/>
-        <v>input2-256-1-3-50-60.xlsx</v>
-      </c>
-      <c r="O8" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v>P1-alone_P2-FL_7.xlsx</v>
-      </c>
-      <c r="P8" s="23">
-        <v>1.8324760595354599</v>
-      </c>
-      <c r="Q8" s="24">
-        <v>0.999999999999997</v>
-      </c>
-      <c r="R8" s="23">
-        <v>0.83247605953546899</v>
-      </c>
-      <c r="S8" s="25">
-        <v>1.77752156719893</v>
-      </c>
-      <c r="T8" s="25">
-        <v>0.94110312500000004</v>
-      </c>
-      <c r="U8" s="25">
-        <v>0.83641844219893502</v>
-      </c>
-      <c r="V8" s="26">
-        <v>0.78943180000351199</v>
-      </c>
-      <c r="W8" s="26">
-        <v>599.45193720001396</v>
-      </c>
-      <c r="X8" s="26">
-        <v>600.24136900001702</v>
-      </c>
-      <c r="BQ8" s="12"/>
-      <c r="EP8" s="12"/>
-      <c r="EW8" s="12"/>
-      <c r="FA8" s="12"/>
-      <c r="IL8" s="12"/>
-      <c r="LK8" s="12"/>
-      <c r="LR8" s="12"/>
-      <c r="LV8" s="12"/>
-    </row>
-    <row r="9" spans="1:16358" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="B9" s="22">
@@ -18048,53 +18047,53 @@
       <c r="M9" s="22">
         <v>60</v>
       </c>
-      <c r="N9" s="21" t="str">
+      <c r="N9" s="23">
+        <v>1.8343130550162201</v>
+      </c>
+      <c r="O9" s="24">
+        <v>0.999999999999999</v>
+      </c>
+      <c r="P9" s="23">
+        <v>0.83431305501622899</v>
+      </c>
+      <c r="Q9" s="25">
+        <v>1.7784626883672201</v>
+      </c>
+      <c r="R9" s="25">
+        <v>0.94094140625004496</v>
+      </c>
+      <c r="S9" s="25">
+        <v>0.83752128211717902</v>
+      </c>
+      <c r="T9" s="26">
+        <v>0.57759890000306702</v>
+      </c>
+      <c r="U9" s="26">
+        <v>599.59585900003003</v>
+      </c>
+      <c r="V9" s="26">
+        <v>600.17345790003299</v>
+      </c>
+      <c r="W9" s="21" t="str">
+        <f>"input"&amp;B9&amp;"-"&amp;E9&amp;"-"&amp;J9&amp;"-"&amp;K9&amp;"-"&amp;L9&amp;"-"&amp;M9&amp;".xlsx"</f>
+        <v>input3-256-1-3-50-60.xlsx</v>
+      </c>
+      <c r="X9" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v>IP_vector_alone_2FL_reopt-c8c.xlsx</v>
+      </c>
+      <c r="BO9" s="12"/>
+      <c r="EN9" s="12"/>
+      <c r="EU9" s="12"/>
+      <c r="EY9" s="12"/>
+      <c r="IJ9" s="12"/>
+      <c r="LI9" s="12"/>
+      <c r="LP9" s="12"/>
+      <c r="LT9" s="12"/>
+    </row>
+    <row r="10" spans="1:16356" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
         <f t="shared" si="0"/>
-        <v>input3-256-1-3-50-60.xlsx</v>
-      </c>
-      <c r="O9" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v>P1-alone_P2-FL_8.xlsx</v>
-      </c>
-      <c r="P9" s="23">
-        <v>1.8343130550162201</v>
-      </c>
-      <c r="Q9" s="24">
-        <v>0.999999999999999</v>
-      </c>
-      <c r="R9" s="23">
-        <v>0.83431305501622899</v>
-      </c>
-      <c r="S9" s="25">
-        <v>1.7784626883672201</v>
-      </c>
-      <c r="T9" s="25">
-        <v>0.94094140625004496</v>
-      </c>
-      <c r="U9" s="25">
-        <v>0.83752128211717902</v>
-      </c>
-      <c r="V9" s="26">
-        <v>0.57759890000306702</v>
-      </c>
-      <c r="W9" s="26">
-        <v>599.59585900003003</v>
-      </c>
-      <c r="X9" s="26">
-        <v>600.17345790003299</v>
-      </c>
-      <c r="BQ9" s="12"/>
-      <c r="EP9" s="12"/>
-      <c r="EW9" s="12"/>
-      <c r="FA9" s="12"/>
-      <c r="IL9" s="12"/>
-      <c r="LK9" s="12"/>
-      <c r="LR9" s="12"/>
-      <c r="LV9" s="12"/>
-    </row>
-    <row r="10" spans="1:16358" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="B10" s="22">
@@ -18133,53 +18132,53 @@
       <c r="M10" s="22">
         <v>60</v>
       </c>
-      <c r="N10" s="21" t="str">
+      <c r="N10" s="23">
+        <v>1.8324772198831201</v>
+      </c>
+      <c r="O10" s="24">
+        <v>0.999999999999997</v>
+      </c>
+      <c r="P10" s="23">
+        <v>0.83247721988312395</v>
+      </c>
+      <c r="Q10" s="25">
+        <v>1.77520842811503</v>
+      </c>
+      <c r="R10" s="25">
+        <v>0.94229531249558496</v>
+      </c>
+      <c r="S10" s="25">
+        <v>0.83291311561944603</v>
+      </c>
+      <c r="T10" s="26">
+        <v>0.62266380000073696</v>
+      </c>
+      <c r="U10" s="26">
+        <v>599.52680149998196</v>
+      </c>
+      <c r="V10" s="26">
+        <v>600.14946529998201</v>
+      </c>
+      <c r="W10" s="21" t="str">
+        <f>"input"&amp;B10&amp;"-"&amp;E10&amp;"-"&amp;J10&amp;"-"&amp;K10&amp;"-"&amp;L10&amp;"-"&amp;M10&amp;".xlsx"</f>
+        <v>input4-256-1-3-50-60.xlsx</v>
+      </c>
+      <c r="X10" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v>IP_vector_alone_2FL_reopt-c9c.xlsx</v>
+      </c>
+      <c r="BO10" s="12"/>
+      <c r="EN10" s="12"/>
+      <c r="EU10" s="12"/>
+      <c r="EY10" s="12"/>
+      <c r="IJ10" s="12"/>
+      <c r="LI10" s="12"/>
+      <c r="LP10" s="12"/>
+      <c r="LT10" s="12"/>
+    </row>
+    <row r="11" spans="1:16356" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
         <f t="shared" si="0"/>
-        <v>input4-256-1-3-50-60.xlsx</v>
-      </c>
-      <c r="O10" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v>P1-alone_P2-FL_9.xlsx</v>
-      </c>
-      <c r="P10" s="23">
-        <v>1.8324772198831201</v>
-      </c>
-      <c r="Q10" s="24">
-        <v>0.999999999999997</v>
-      </c>
-      <c r="R10" s="23">
-        <v>0.83247721988312395</v>
-      </c>
-      <c r="S10" s="25">
-        <v>1.77520842811503</v>
-      </c>
-      <c r="T10" s="25">
-        <v>0.94229531249558496</v>
-      </c>
-      <c r="U10" s="25">
-        <v>0.83291311561944603</v>
-      </c>
-      <c r="V10" s="26">
-        <v>0.62266380000073696</v>
-      </c>
-      <c r="W10" s="26">
-        <v>599.52680149998196</v>
-      </c>
-      <c r="X10" s="26">
-        <v>600.14946529998201</v>
-      </c>
-      <c r="BQ10" s="12"/>
-      <c r="EP10" s="12"/>
-      <c r="EW10" s="12"/>
-      <c r="FA10" s="12"/>
-      <c r="IL10" s="12"/>
-      <c r="LK10" s="12"/>
-      <c r="LR10" s="12"/>
-      <c r="LV10" s="12"/>
-    </row>
-    <row r="11" spans="1:16358" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
-        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="B11" s="22">
@@ -18218,49 +18217,49 @@
       <c r="M11" s="22">
         <v>60</v>
       </c>
-      <c r="N11" s="21" t="str">
-        <f t="shared" si="0"/>
+      <c r="N11" s="23">
+        <v>1.8339301599953599</v>
+      </c>
+      <c r="O11" s="24">
+        <v>0.999999999999998</v>
+      </c>
+      <c r="P11" s="23">
+        <v>0.83393015999536602</v>
+      </c>
+      <c r="Q11" s="25">
+        <v>1.8165570244771401</v>
+      </c>
+      <c r="R11" s="25">
+        <v>0.96309218749999703</v>
+      </c>
+      <c r="S11" s="25">
+        <v>0.85346483697714803</v>
+      </c>
+      <c r="T11" s="26">
+        <v>0.78711340000154395</v>
+      </c>
+      <c r="U11" s="26">
+        <v>599.42067090001296</v>
+      </c>
+      <c r="V11" s="26">
+        <v>600.20778430001496</v>
+      </c>
+      <c r="W11" s="21" t="str">
+        <f>"input"&amp;B11&amp;"-"&amp;E11&amp;"-"&amp;J11&amp;"-"&amp;K11&amp;"-"&amp;L11&amp;"-"&amp;M11&amp;".xlsx"</f>
         <v>input5-256-1-3-50-60.xlsx</v>
       </c>
-      <c r="O11" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v>P1-alone_P2-FL_10.xlsx</v>
-      </c>
-      <c r="P11" s="23">
-        <v>1.8339301599953599</v>
-      </c>
-      <c r="Q11" s="24">
-        <v>0.999999999999998</v>
-      </c>
-      <c r="R11" s="23">
-        <v>0.83393015999536602</v>
-      </c>
-      <c r="S11" s="25">
-        <v>1.8165570244771401</v>
-      </c>
-      <c r="T11" s="25">
-        <v>0.96309218749999703</v>
-      </c>
-      <c r="U11" s="25">
-        <v>0.85346483697714803</v>
-      </c>
-      <c r="V11" s="26">
-        <v>0.78711340000154395</v>
-      </c>
-      <c r="W11" s="26">
-        <v>599.42067090001296</v>
-      </c>
-      <c r="X11" s="26">
-        <v>600.20778430001496</v>
-      </c>
-      <c r="BQ11" s="12"/>
-      <c r="EP11" s="12"/>
-      <c r="EW11" s="12"/>
-      <c r="FA11" s="12"/>
-      <c r="IL11" s="12"/>
-      <c r="LK11" s="12"/>
-      <c r="LR11" s="12"/>
-      <c r="LV11" s="12"/>
+      <c r="X11" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v>IP_vector_alone_2FL_reopt-c10c.xlsx</v>
+      </c>
+      <c r="BO11" s="12"/>
+      <c r="EN11" s="12"/>
+      <c r="EU11" s="12"/>
+      <c r="EY11" s="12"/>
+      <c r="IJ11" s="12"/>
+      <c r="LI11" s="12"/>
+      <c r="LP11" s="12"/>
+      <c r="LT11" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>